<commit_message>
Add _pm_paym_filter feature and fix S00026 over-extraction for 4 DTCDs
세션33 변경사항:
- generate_intermediate.py: _pm_paym_filter 신규 기능 (PM sub_type 키워드→PAYM 타입 라우팅)
  - 예: {거치형: [""], 적립형: ["N","X"]} → 분납/거치형 ITCD별 행 분리
- generate_intermediate.py: is_galsin 추가 (MIN_AG≥25 갱신형 행 건강체 PM 공유)
- product_exceptions.json: 1228/1629/1758/2042 S00026 설정 추가
  - 1228/1629: _sub_type_filter + _max_ag_limit_by_paym (기본형 필터 + MAX_AG 상한)
  - 1758/2042: _pm_paym_filter (적립형/거치형 PAYM 라우팅)

결과: S00026 중간검증 PASS 39→43 (+4), 일치 79→96 (+17), 과잉추출 23→6

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/existing/판매중_납입주기정보_0312.xlsx
+++ b/data/existing/판매중_납입주기정보_0312.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -47,7 +47,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +84,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -103,6 +108,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>